<commit_message>
bug fix at reading product_master excel file + product-line compatibility matrix to excel + side excel files for minimal use of HTL6.
</commit_message>
<xml_diff>
--- a/backend/domain/ProductionPlanning_v6.xlsx
+++ b/backend/domain/ProductionPlanning_v6.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alex\Master\2026 SS\Masterarbeit\phase 3\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alex\Master\2026 SS\Masterarbeit\phase 3\backend\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF1A32EF-B266-40DD-BD7C-49378691A77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8161686F-96D7-4669-A62C-9D853C1E9254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="580" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OEE" sheetId="15" r:id="rId1"/>
@@ -26,8 +26,7 @@
     <sheet name="CustomerDemandKanban" sheetId="10" r:id="rId11"/>
     <sheet name="KanbanCardsSetup" sheetId="9" r:id="rId12"/>
     <sheet name="KanbanConfig" sheetId="12" r:id="rId13"/>
-    <sheet name="SupermInState" sheetId="11" r:id="rId14"/>
-    <sheet name="README" sheetId="8" r:id="rId15"/>
+    <sheet name="README" sheetId="8" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">CustomerDemand!$A$3:$E$8</definedName>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="326">
   <si>
     <t>PROCESS PARAMETERS</t>
   </si>
@@ -649,13 +648,7 @@
     <t>Time</t>
   </si>
   <si>
-    <t>InitialCards</t>
-  </si>
-  <si>
     <t>InitialPcsPartial</t>
-  </si>
-  <si>
-    <t>InitialCards = full batches (cards) sitting in the line's supermarket at t=0. InitialPcsPartial = leftover pcs not yet forming a full card (0-BatchSize-1).</t>
   </si>
   <si>
     <t>BatchSize = pcs per card (defaults to 50; Packaging sheet PK1 = 25 pcs/pack, review consistency)
@@ -1477,9 +1470,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1502,9 +1498,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1780,15 +1773,15 @@
   <sheetData>
     <row r="1" spans="1:4" ht="16.899999999999999" x14ac:dyDescent="0.45">
       <c r="A1" s="44" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B1" s="45"/>
       <c r="C1" s="45"/>
       <c r="D1" s="45"/>
     </row>
     <row r="2" spans="1:4" ht="78.400000000000006" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="57" t="s">
-        <v>324</v>
+      <c r="A2" s="46" t="s">
+        <v>322</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -1799,13 +1792,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>325</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
@@ -2133,37 +2126,37 @@
       <c r="E1" s="44"/>
     </row>
     <row r="2" spans="1:5" ht="29.35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="50" t="s">
-        <v>211</v>
-      </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
+      <c r="A2" s="51" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
     </row>
     <row r="3" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A3" s="36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B3" s="36" t="s">
         <v>202</v>
       </c>
       <c r="C3" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="D3" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="E3" s="36" t="s">
         <v>227</v>
-      </c>
-      <c r="D3" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="E3" s="36" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="37" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C4" s="38" t="s">
         <v>87</v>
@@ -2172,15 +2165,15 @@
         <v>1000</v>
       </c>
       <c r="E4" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="37" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C5" s="38" t="s">
         <v>178</v>
@@ -2189,15 +2182,15 @@
         <v>500</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="37" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C6" s="38" t="s">
         <v>89</v>
@@ -2206,15 +2199,15 @@
         <v>1600</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="37" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C7" s="38" t="s">
         <v>176</v>
@@ -2223,15 +2216,15 @@
         <v>200</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="37" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C8" s="38" t="s">
         <v>85</v>
@@ -2240,15 +2233,15 @@
         <v>2800</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="37" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C9" s="38" t="s">
         <v>165</v>
@@ -2257,15 +2250,15 @@
         <v>1000</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C10" s="38" t="s">
         <v>85</v>
@@ -2274,15 +2267,15 @@
         <v>200</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C11" s="38" t="s">
         <v>188</v>
@@ -2291,15 +2284,15 @@
         <v>1600</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C12" s="38" t="s">
         <v>164</v>
@@ -2308,15 +2301,15 @@
         <v>600</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C13" s="38" t="s">
         <v>166</v>
@@ -2325,15 +2318,15 @@
         <v>3000</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="37" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C14" s="38" t="s">
         <v>147</v>
@@ -2342,15 +2335,15 @@
         <v>600</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="37" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C15" s="38" t="s">
         <v>85</v>
@@ -2359,15 +2352,15 @@
         <v>400</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="37" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C16" s="38" t="s">
         <v>177</v>
@@ -2376,15 +2369,15 @@
         <v>1200</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="37" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C17" s="38" t="s">
         <v>162</v>
@@ -2393,15 +2386,15 @@
         <v>1200</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="37" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C18" s="38" t="s">
         <v>176</v>
@@ -2410,15 +2403,15 @@
         <v>2200</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="37" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C19" s="38" t="s">
         <v>88</v>
@@ -2427,15 +2420,15 @@
         <v>2400</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="37" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C20" s="38" t="s">
         <v>177</v>
@@ -2444,15 +2437,15 @@
         <v>1200</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" s="37" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C21" s="38" t="s">
         <v>89</v>
@@ -2461,15 +2454,15 @@
         <v>1000</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" s="37" t="s">
+        <v>279</v>
+      </c>
+      <c r="B22" s="37" t="s">
         <v>281</v>
-      </c>
-      <c r="B22" s="37" t="s">
-        <v>283</v>
       </c>
       <c r="C22" s="38" t="s">
         <v>84</v>
@@ -2478,15 +2471,15 @@
         <v>800</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" s="37" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C23" s="38" t="s">
         <v>87</v>
@@ -2495,15 +2488,15 @@
         <v>1000</v>
       </c>
       <c r="E23" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" s="37" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C24" s="38" t="s">
         <v>166</v>
@@ -2512,15 +2505,15 @@
         <v>3000</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" s="37" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B25" s="37" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C25" s="38" t="s">
         <v>85</v>
@@ -2529,15 +2522,15 @@
         <v>1600</v>
       </c>
       <c r="E25" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" s="37" t="s">
+        <v>284</v>
+      </c>
+      <c r="B26" s="37" t="s">
         <v>286</v>
-      </c>
-      <c r="B26" s="37" t="s">
-        <v>288</v>
       </c>
       <c r="C26" s="38" t="s">
         <v>178</v>
@@ -2546,15 +2539,15 @@
         <v>1600</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" s="37" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B27" s="37" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C27" s="38" t="s">
         <v>156</v>
@@ -2563,15 +2556,15 @@
         <v>900</v>
       </c>
       <c r="E27" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" s="37" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C28" s="38" t="s">
         <v>152</v>
@@ -2580,15 +2573,15 @@
         <v>2600</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" s="37" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B29" s="37" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C29" s="38" t="s">
         <v>186</v>
@@ -2597,15 +2590,15 @@
         <v>1000</v>
       </c>
       <c r="E29" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" s="37" t="s">
+        <v>290</v>
+      </c>
+      <c r="B30" s="37" t="s">
         <v>292</v>
-      </c>
-      <c r="B30" s="37" t="s">
-        <v>294</v>
       </c>
       <c r="C30" s="38" t="s">
         <v>156</v>
@@ -2614,15 +2607,15 @@
         <v>2400</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" s="37" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B31" s="37" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C31" s="38" t="s">
         <v>187</v>
@@ -2631,15 +2624,15 @@
         <v>2200</v>
       </c>
       <c r="E31" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" s="37" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B32" s="37" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C32" s="38" t="s">
         <v>152</v>
@@ -2648,15 +2641,15 @@
         <v>800</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" s="37" t="s">
+        <v>294</v>
+      </c>
+      <c r="B33" s="37" t="s">
         <v>296</v>
-      </c>
-      <c r="B33" s="37" t="s">
-        <v>298</v>
       </c>
       <c r="C33" s="38" t="s">
         <v>83</v>
@@ -2665,15 +2658,15 @@
         <v>600</v>
       </c>
       <c r="E33" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" s="37" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B34" s="37" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C34" s="38" t="s">
         <v>148</v>
@@ -2682,15 +2675,15 @@
         <v>200</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" s="37" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B35" s="37" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C35" s="38" t="s">
         <v>166</v>
@@ -2699,15 +2692,15 @@
         <v>2600</v>
       </c>
       <c r="E35" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" s="37" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B36" s="37" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C36" s="38" t="s">
         <v>162</v>
@@ -2716,15 +2709,15 @@
         <v>1200</v>
       </c>
       <c r="E36" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" s="37" t="s">
+        <v>299</v>
+      </c>
+      <c r="B37" s="37" t="s">
         <v>301</v>
-      </c>
-      <c r="B37" s="37" t="s">
-        <v>303</v>
       </c>
       <c r="C37" s="38" t="s">
         <v>89</v>
@@ -2733,15 +2726,15 @@
         <v>2000</v>
       </c>
       <c r="E37" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" s="37" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B38" s="37" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C38" s="38" t="s">
         <v>178</v>
@@ -2750,15 +2743,15 @@
         <v>400</v>
       </c>
       <c r="E38" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" s="37" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B39" s="37" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C39" s="38" t="s">
         <v>88</v>
@@ -2767,15 +2760,15 @@
         <v>1000</v>
       </c>
       <c r="E39" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" s="37" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B40" s="37" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C40" s="38" t="s">
         <v>90</v>
@@ -2784,7 +2777,7 @@
         <v>800</v>
       </c>
       <c r="E40" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -2816,27 +2809,27 @@
     </row>
     <row r="2" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A2" s="36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B2" s="36" t="s">
         <v>202</v>
       </c>
       <c r="C2" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="D2" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="E2" s="36" t="s">
         <v>227</v>
-      </c>
-      <c r="D2" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="E2" s="36" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="37" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C3" s="38" t="s">
         <v>190</v>
@@ -2845,15 +2838,15 @@
         <v>3000</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="37" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C4" s="38" t="s">
         <v>180</v>
@@ -2862,15 +2855,15 @@
         <v>2600</v>
       </c>
       <c r="E4" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="37" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C5" s="38" t="s">
         <v>195</v>
@@ -2879,15 +2872,15 @@
         <v>3200</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="37" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C6" s="38" t="s">
         <v>160</v>
@@ -2896,15 +2889,15 @@
         <v>3000</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="37" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C7" s="38" t="s">
         <v>190</v>
@@ -2913,15 +2906,15 @@
         <v>1200</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="37" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C8" s="38" t="s">
         <v>190</v>
@@ -2930,15 +2923,15 @@
         <v>3000</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C9" s="38" t="s">
         <v>190</v>
@@ -2947,15 +2940,15 @@
         <v>3000</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C10" s="38" t="s">
         <v>180</v>
@@ -2964,15 +2957,15 @@
         <v>2400</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="37" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C11" s="38" t="s">
         <v>168</v>
@@ -2981,15 +2974,15 @@
         <v>2600</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="37" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C12" s="38" t="s">
         <v>180</v>
@@ -2998,15 +2991,15 @@
         <v>1000</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="37" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C13" s="38" t="s">
         <v>180</v>
@@ -3015,15 +3008,15 @@
         <v>3000</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="37" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C14" s="38" t="s">
         <v>168</v>
@@ -3032,15 +3025,15 @@
         <v>2800</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="37" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C15" s="38" t="s">
         <v>180</v>
@@ -3049,15 +3042,15 @@
         <v>1600</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="37" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C16" s="38" t="s">
         <v>190</v>
@@ -3066,15 +3059,15 @@
         <v>1400</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="37" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C17" s="38" t="s">
         <v>190</v>
@@ -3083,15 +3076,15 @@
         <v>3600</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="37" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C18" s="38" t="s">
         <v>160</v>
@@ -3100,15 +3093,15 @@
         <v>3000</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="37" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C19" s="38" t="s">
         <v>160</v>
@@ -3117,15 +3110,15 @@
         <v>1600</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="37" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C20" s="38" t="s">
         <v>190</v>
@@ -3134,15 +3127,15 @@
         <v>5000</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="37" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C21" s="38" t="s">
         <v>180</v>
@@ -3151,15 +3144,15 @@
         <v>2000</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="37" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C22" s="38" t="s">
         <v>180</v>
@@ -3168,15 +3161,15 @@
         <v>3400</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="37" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C23" s="38" t="s">
         <v>190</v>
@@ -3185,15 +3178,15 @@
         <v>3400</v>
       </c>
       <c r="E23" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="37" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C24" s="38" t="s">
         <v>180</v>
@@ -3202,15 +3195,15 @@
         <v>1600</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="37" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B25" s="37" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C25" s="38" t="s">
         <v>160</v>
@@ -3219,15 +3212,15 @@
         <v>3000</v>
       </c>
       <c r="E25" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="37" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C26" s="38" t="s">
         <v>180</v>
@@ -3236,15 +3229,15 @@
         <v>2000</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="37" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B27" s="37" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C27" s="38" t="s">
         <v>180</v>
@@ -3253,15 +3246,15 @@
         <v>800</v>
       </c>
       <c r="E27" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="37" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C28" s="38" t="s">
         <v>195</v>
@@ -3270,15 +3263,15 @@
         <v>2800</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="37" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B29" s="37" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C29" s="38" t="s">
         <v>190</v>
@@ -3287,15 +3280,15 @@
         <v>3000</v>
       </c>
       <c r="E29" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="37" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B30" s="37" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C30" s="38" t="s">
         <v>190</v>
@@ -3304,15 +3297,15 @@
         <v>3000</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="37" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B31" s="37" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C31" s="38" t="s">
         <v>180</v>
@@ -3321,15 +3314,15 @@
         <v>3400</v>
       </c>
       <c r="E31" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="37" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B32" s="37" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C32" s="38" t="s">
         <v>195</v>
@@ -3338,15 +3331,15 @@
         <v>200</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="37" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B33" s="37" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C33" s="38" t="s">
         <v>190</v>
@@ -3355,15 +3348,15 @@
         <v>4000</v>
       </c>
       <c r="E33" s="37" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="37" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B34" s="37" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C34" s="38" t="s">
         <v>180</v>
@@ -3372,7 +3365,7 @@
         <v>4000</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -3412,7 +3405,7 @@
         <v>17</v>
       </c>
       <c r="H1" s="34" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="I1" s="30"/>
     </row>
@@ -3427,7 +3420,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H2" s="25"/>
     </row>
@@ -3442,7 +3435,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.45">
@@ -3456,7 +3449,7 @@
         <v>4</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
@@ -3470,7 +3463,7 @@
         <v>4</v>
       </c>
       <c r="F5" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
@@ -3484,7 +3477,7 @@
         <v>4</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
@@ -3498,7 +3491,7 @@
         <v>4</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
@@ -3512,10 +3505,10 @@
         <v>4</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.45">
@@ -3529,10 +3522,10 @@
         <v>4</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.45">
@@ -3546,7 +3539,7 @@
         <v>4</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.45">
@@ -3560,10 +3553,10 @@
         <v>4</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.45">
@@ -3577,7 +3570,7 @@
         <v>4</v>
       </c>
       <c r="D12" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.45">
@@ -3591,10 +3584,10 @@
         <v>4</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.45">
@@ -3608,7 +3601,7 @@
         <v>4</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.45">
@@ -3622,7 +3615,7 @@
         <v>4</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.45">
@@ -3636,7 +3629,7 @@
         <v>4</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.45">
@@ -3650,7 +3643,7 @@
         <v>4</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.45">
@@ -3664,7 +3657,7 @@
         <v>4</v>
       </c>
       <c r="D18" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.45">
@@ -3678,13 +3671,13 @@
         <v>4</v>
       </c>
       <c r="D19" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.45">
@@ -3698,7 +3691,7 @@
         <v>4</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.45">
@@ -3712,7 +3705,7 @@
         <v>4</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.45">
@@ -3726,13 +3719,13 @@
         <v>4</v>
       </c>
       <c r="D22" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F22" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.45">
@@ -3746,7 +3739,7 @@
         <v>4</v>
       </c>
       <c r="D23" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.45">
@@ -3760,7 +3753,7 @@
         <v>4</v>
       </c>
       <c r="D24" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.45">
@@ -3774,7 +3767,7 @@
         <v>4</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.45">
@@ -3788,7 +3781,7 @@
         <v>4</v>
       </c>
       <c r="D26" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.45">
@@ -3802,7 +3795,7 @@
         <v>4</v>
       </c>
       <c r="F27" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.45">
@@ -3816,7 +3809,7 @@
         <v>4</v>
       </c>
       <c r="D28" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.45">
@@ -3830,10 +3823,10 @@
         <v>4</v>
       </c>
       <c r="D29" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F29" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.45">
@@ -3847,7 +3840,7 @@
         <v>4</v>
       </c>
       <c r="D30" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.45">
@@ -3861,7 +3854,7 @@
         <v>4</v>
       </c>
       <c r="E31" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.45">
@@ -3875,7 +3868,7 @@
         <v>4</v>
       </c>
       <c r="D32" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.45">
@@ -3889,10 +3882,10 @@
         <v>4</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F33" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.45">
@@ -3906,10 +3899,10 @@
         <v>4</v>
       </c>
       <c r="E34" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F34" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.45">
@@ -3923,13 +3916,13 @@
         <v>4</v>
       </c>
       <c r="D35" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E35" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F35" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.45">
@@ -3943,10 +3936,10 @@
         <v>4</v>
       </c>
       <c r="D36" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E36" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.45">
@@ -3960,10 +3953,10 @@
         <v>4</v>
       </c>
       <c r="D37" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F37" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.45">
@@ -3977,10 +3970,10 @@
         <v>4</v>
       </c>
       <c r="E38" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F38" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.45">
@@ -3994,10 +3987,10 @@
         <v>4</v>
       </c>
       <c r="D39" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E39" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.45">
@@ -4011,10 +4004,10 @@
         <v>4</v>
       </c>
       <c r="D40" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E40" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.45">
@@ -4028,10 +4021,10 @@
         <v>4</v>
       </c>
       <c r="D41" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E41" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.45">
@@ -4045,10 +4038,10 @@
         <v>4</v>
       </c>
       <c r="D42" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E42" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.45">
@@ -4062,10 +4055,10 @@
         <v>4</v>
       </c>
       <c r="D43" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F43" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.45">
@@ -4079,10 +4072,10 @@
         <v>4</v>
       </c>
       <c r="E44" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F44" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.45">
@@ -4096,10 +4089,10 @@
         <v>4</v>
       </c>
       <c r="E45" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F45" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.45">
@@ -4113,10 +4106,10 @@
         <v>4</v>
       </c>
       <c r="D46" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F46" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.45">
@@ -4130,10 +4123,10 @@
         <v>4</v>
       </c>
       <c r="E47" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F47" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.45">
@@ -4147,10 +4140,10 @@
         <v>4</v>
       </c>
       <c r="D48" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F48" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.45">
@@ -4164,10 +4157,10 @@
         <v>4</v>
       </c>
       <c r="D49" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F49" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.45">
@@ -4181,10 +4174,10 @@
         <v>4</v>
       </c>
       <c r="D50" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F50" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.45">
@@ -4198,10 +4191,10 @@
         <v>4</v>
       </c>
       <c r="D51" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E51" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.45">
@@ -4215,10 +4208,10 @@
         <v>4</v>
       </c>
       <c r="D52" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E52" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.45">
@@ -4232,10 +4225,10 @@
         <v>4</v>
       </c>
       <c r="E53" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F53" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.45">
@@ -4249,7 +4242,7 @@
         <v>4</v>
       </c>
       <c r="D54" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.45">
@@ -4263,10 +4256,10 @@
         <v>4</v>
       </c>
       <c r="D55" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E55" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.45">
@@ -4280,7 +4273,7 @@
         <v>4</v>
       </c>
       <c r="D56" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.45">
@@ -4294,10 +4287,10 @@
         <v>4</v>
       </c>
       <c r="E57" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F57" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.45">
@@ -4311,10 +4304,10 @@
         <v>4</v>
       </c>
       <c r="D58" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E58" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.45">
@@ -4328,10 +4321,10 @@
         <v>4</v>
       </c>
       <c r="D59" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F59" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.45">
@@ -4345,10 +4338,10 @@
         <v>4</v>
       </c>
       <c r="E60" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F60" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.45">
@@ -4362,10 +4355,10 @@
         <v>4</v>
       </c>
       <c r="D61" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E61" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.45">
@@ -4379,10 +4372,10 @@
         <v>4</v>
       </c>
       <c r="E62" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F62" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.45">
@@ -4396,10 +4389,10 @@
         <v>4</v>
       </c>
       <c r="D63" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E63" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.45">
@@ -4413,7 +4406,7 @@
         <v>4</v>
       </c>
       <c r="F64" s="31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -4443,35 +4436,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="32" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B2" s="31">
         <v>50</v>
       </c>
       <c r="C2" s="31" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="32" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B3" s="31">
         <v>30</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="32" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B4" s="31">
         <v>25</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -4480,138 +4473,6 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="6" max="6" width="90" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A1" s="29" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="29" t="s">
-        <v>144</v>
-      </c>
-      <c r="C1" s="29" t="s">
-        <v>203</v>
-      </c>
-      <c r="D1" s="29" t="s">
-        <v>204</v>
-      </c>
-      <c r="F1" s="30" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>190</v>
-      </c>
-      <c r="C2">
-        <v>19</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>180</v>
-      </c>
-      <c r="C3">
-        <v>12</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C4">
-        <v>19</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
-        <v>190</v>
-      </c>
-      <c r="C5">
-        <v>19</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" t="s">
-        <v>180</v>
-      </c>
-      <c r="C6">
-        <v>12</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>160</v>
-      </c>
-      <c r="C7">
-        <v>14</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>195</v>
-      </c>
-      <c r="C8">
-        <v>24</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C18"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -4726,46 +4587,46 @@
     </row>
     <row r="11" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="46" t="s">
+      <c r="A13" s="48" t="s">
         <v>138</v>
       </c>
       <c r="B13" s="47"/>
       <c r="C13" s="47"/>
     </row>
     <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="51" t="s">
+      <c r="A14" s="52" t="s">
         <v>139</v>
       </c>
       <c r="B14" s="47"/>
-      <c r="C14" s="52"/>
+      <c r="C14" s="53"/>
     </row>
     <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="55" t="s">
+      <c r="A15" s="56" t="s">
         <v>140</v>
       </c>
       <c r="B15" s="47"/>
-      <c r="C15" s="52"/>
+      <c r="C15" s="53"/>
     </row>
     <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="56" t="s">
+      <c r="A16" s="57" t="s">
         <v>141</v>
       </c>
       <c r="B16" s="47"/>
-      <c r="C16" s="52"/>
+      <c r="C16" s="53"/>
     </row>
     <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="53" t="s">
+      <c r="A17" s="54" t="s">
         <v>142</v>
       </c>
       <c r="B17" s="47"/>
-      <c r="C17" s="52"/>
+      <c r="C17" s="53"/>
     </row>
     <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="54" t="s">
+      <c r="A18" s="55" t="s">
         <v>143</v>
       </c>
       <c r="B18" s="47"/>
-      <c r="C18" s="52"/>
+      <c r="C18" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -4806,8 +4667,8 @@
       <c r="F1" s="45"/>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="46" t="s">
-        <v>322</v>
+      <c r="A2" s="48" t="s">
+        <v>320</v>
       </c>
       <c r="B2" s="47"/>
       <c r="C2" s="47"/>
@@ -5210,7 +5071,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="48" t="s">
+      <c r="A21" s="49" t="s">
         <v>18</v>
       </c>
       <c r="B21" s="45"/>
@@ -5241,7 +5102,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.45">
       <c r="A1" s="44" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B1" s="44"/>
       <c r="C1" s="45"/>
@@ -5251,18 +5112,18 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B3" s="43">
         <v>0.25</v>
@@ -5273,7 +5134,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="6" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B4" s="43">
         <v>0.58333333333333337</v>
@@ -5284,7 +5145,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B5" s="43">
         <v>0.91666666666666663</v>
@@ -5298,19 +5159,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>262</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
@@ -5321,16 +5182,16 @@
         <v>46266</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
@@ -5341,16 +5202,16 @@
         <v>46267</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
@@ -5361,16 +5222,16 @@
         <v>46268</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
@@ -5381,16 +5242,16 @@
         <v>46269</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
@@ -5401,10 +5262,10 @@
         <v>46270</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -5417,7 +5278,7 @@
         <v>46271</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
@@ -5431,16 +5292,16 @@
         <v>46272</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
@@ -5451,16 +5312,16 @@
         <v>46273</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
@@ -5471,16 +5332,16 @@
         <v>46274</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
@@ -5491,16 +5352,16 @@
         <v>46275</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.45">
@@ -5511,16 +5372,16 @@
         <v>46276</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.45">
@@ -5531,10 +5392,10 @@
         <v>46277</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -5547,7 +5408,7 @@
         <v>46278</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
@@ -5561,16 +5422,16 @@
         <v>46279</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.45">
@@ -5581,16 +5442,16 @@
         <v>46280</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.45">
@@ -5601,16 +5462,16 @@
         <v>46281</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.45">
@@ -5621,16 +5482,16 @@
         <v>46266</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.45">
@@ -5641,16 +5502,16 @@
         <v>46267</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.45">
@@ -5661,16 +5522,16 @@
         <v>46268</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.45">
@@ -5681,16 +5542,16 @@
         <v>46269</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.45">
@@ -5701,10 +5562,10 @@
         <v>46270</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
@@ -5717,7 +5578,7 @@
         <v>46271</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
@@ -5731,16 +5592,16 @@
         <v>46272</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.45">
@@ -5751,16 +5612,16 @@
         <v>46273</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.45">
@@ -5771,16 +5632,16 @@
         <v>46274</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.45">
@@ -5791,16 +5652,16 @@
         <v>46275</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.45">
@@ -5811,16 +5672,16 @@
         <v>46276</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.45">
@@ -5831,10 +5692,10 @@
         <v>46277</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
@@ -5847,7 +5708,7 @@
         <v>46278</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
@@ -5861,16 +5722,16 @@
         <v>46279</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.45">
@@ -5881,16 +5742,16 @@
         <v>46280</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.45">
@@ -5901,16 +5762,16 @@
         <v>46281</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.45">
@@ -5921,16 +5782,16 @@
         <v>46266</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.45">
@@ -5941,16 +5802,16 @@
         <v>46267</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.45">
@@ -5961,16 +5822,16 @@
         <v>46268</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.45">
@@ -5981,16 +5842,16 @@
         <v>46269</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.45">
@@ -6001,10 +5862,10 @@
         <v>46270</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
@@ -6017,7 +5878,7 @@
         <v>46271</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
@@ -6031,16 +5892,16 @@
         <v>46272</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.45">
@@ -6051,16 +5912,16 @@
         <v>46273</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.45">
@@ -6071,16 +5932,16 @@
         <v>46274</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.45">
@@ -6091,16 +5952,16 @@
         <v>46275</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.45">
@@ -6111,16 +5972,16 @@
         <v>46276</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.45">
@@ -6131,10 +5992,10 @@
         <v>46277</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
@@ -6147,7 +6008,7 @@
         <v>46278</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
@@ -6161,16 +6022,16 @@
         <v>46279</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.45">
@@ -6181,16 +6042,16 @@
         <v>46280</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.45">
@@ -6201,16 +6062,16 @@
         <v>46281</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -6244,8 +6105,8 @@
       <c r="C1" s="45"/>
       <c r="D1" s="45"/>
       <c r="E1" s="45"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
       <c r="H1" s="45"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -6565,15 +6426,15 @@
       <c r="H14" s="15"/>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="48" t="s">
+      <c r="A16" s="49" t="s">
         <v>43</v>
       </c>
       <c r="B16" s="45"/>
       <c r="C16" s="45"/>
       <c r="D16" s="45"/>
       <c r="E16" s="45"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="49"/>
+      <c r="F16" s="50"/>
+      <c r="G16" s="50"/>
       <c r="H16" s="45"/>
     </row>
   </sheetData>
@@ -7213,7 +7074,7 @@
       <c r="G5" s="3"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A7" s="48" t="s">
+      <c r="A7" s="49" t="s">
         <v>80</v>
       </c>
       <c r="B7" s="45"/>
@@ -7250,22 +7111,22 @@
         <v>2</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C1" s="29" t="s">
         <v>45</v>
       </c>
       <c r="D1" s="29" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E1" s="29" t="s">
         <v>144</v>
       </c>
       <c r="F1" s="29" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="G1" s="29" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
@@ -7276,7 +7137,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D2">
         <v>10</v>
@@ -7299,7 +7160,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -7322,7 +7183,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D4">
         <v>12</v>
@@ -7345,7 +7206,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D5">
         <v>10</v>
@@ -7368,7 +7229,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D6">
         <v>10</v>
@@ -7388,10 +7249,10 @@
         <v>8</v>
       </c>
       <c r="B7" s="31">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D7">
         <v>10</v>
@@ -7408,10 +7269,10 @@
         <v>8</v>
       </c>
       <c r="B8" s="31">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D8">
         <v>10</v>
@@ -7431,7 +7292,7 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D9">
         <v>10</v>
@@ -7454,7 +7315,7 @@
         <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D10">
         <v>10</v>
@@ -7477,7 +7338,7 @@
         <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D11">
         <v>12</v>
@@ -7497,10 +7358,10 @@
         <v>16</v>
       </c>
       <c r="B12" s="31">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D12">
         <v>10</v>
@@ -7517,10 +7378,10 @@
         <v>16</v>
       </c>
       <c r="B13" s="31">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D13">
         <v>10</v>
@@ -7540,7 +7401,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D14">
         <v>10</v>
@@ -7563,7 +7424,7 @@
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D15">
         <v>10</v>
@@ -7586,7 +7447,7 @@
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D16">
         <v>12</v>
@@ -7609,7 +7470,7 @@
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D17">
         <v>12</v>
@@ -7632,7 +7493,7 @@
         <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D18">
         <v>10</v>
@@ -7652,7 +7513,7 @@
         <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D19">
         <v>10</v>

</xml_diff>